<commit_message>
Add NHL/Soccer status cards, remove IP from hero, fix pending state
</commit_message>
<xml_diff>
--- a/NHL/step9_nhl_tickets.xlsx
+++ b/NHL/step9_nhl_tickets.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-06 22:09 UTC</t>
+          <t>Generated: 2026-03-07 17:17 UTC</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Combined Confidence: 9428.2500 (942825.0%)</t>
+          <t>Combined Confidence: 9273.4400 (927344.0%)</t>
         </is>
       </c>
     </row>
@@ -575,12 +575,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
@@ -617,12 +617,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
@@ -633,7 +633,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Combined Confidence: 9233.2500 (923325.0%)</t>
+          <t>Combined Confidence: 9263.7600 (926376.0%)</t>
         </is>
       </c>
     </row>
@@ -724,12 +724,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr"/>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
@@ -766,23 +766,23 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
@@ -809,7 +809,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Combined Confidence: 9157.4900 (915749.0%)</t>
+          <t>Combined Confidence: 9168.0600 (916806.0%)</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
@@ -915,23 +915,23 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Combined Confidence: 9096.7500 (909675.0%)</t>
+          <t>Combined Confidence: 9128.2400 (912824.0%)</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr"/>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="H21" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="H22" s="4" t="n">
-        <v>93.3</v>
+        <v>94.3</v>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Combined Confidence: 9022.1100 (902211.0%)</t>
+          <t>Combined Confidence: 9070.1600 (907016.0%)</t>
         </is>
       </c>
     </row>
@@ -1171,12 +1171,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>96.7</v>
+        <v>96.8</v>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
@@ -1213,18 +1213,18 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>93.3</v>
+        <v>93.7</v>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-06 22:09 UTC</t>
+          <t>Generated: 2026-03-07 17:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Combined Confidence: 892855.2750 (89285527.5%)</t>
+          <t>Combined Confidence: 887468.2080 (88746820.8%)</t>
         </is>
       </c>
     </row>
@@ -1357,12 +1357,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
@@ -1399,12 +1399,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -1441,23 +1441,23 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Combined Confidence: 879655.7250 (87965572.5%)</t>
+          <t>Combined Confidence: 874485.3920 (87448539.2%)</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>93.3</v>
+        <v>94.3</v>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Combined Confidence: 870227.4750 (87022747.5%)</t>
+          <t>Combined Confidence: 873572.5680 (87357256.8%)</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
@@ -1781,12 +1781,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="H19" s="4" t="n">
-        <v>96.7</v>
+        <v>95.7</v>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
@@ -1823,12 +1823,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Wyatt Johnston</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="H20" s="4" t="n">
-        <v>92.3</v>
+        <v>94.3</v>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Combined Confidence: 862684.8750 (86268487.5%)</t>
+          <t>Combined Confidence: 868921.3280 (86892132.8%)</t>
         </is>
       </c>
     </row>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H24" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
@@ -1972,12 +1972,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="H25" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
@@ -2014,23 +2014,23 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Seth Jarvis</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -2039,7 +2039,7 @@
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>91.5</v>
+        <v>93.7</v>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Combined Confidence: 862684.8750 (86268487.5%)</t>
+          <t>Combined Confidence: 868014.3120 (86801431.2%)</t>
         </is>
       </c>
     </row>
@@ -2121,12 +2121,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
@@ -2163,12 +2163,12 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr"/>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="H31" s="4" t="n">
-        <v>96.7</v>
+        <v>95.7</v>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
@@ -2205,12 +2205,12 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Kirill Kaprizov</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>91.5</v>
+        <v>93.7</v>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-06 22:09 UTC</t>
+          <t>Generated: 2026-03-07 17:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Combined Confidence: 83303397.1575 (8330339715.8%)</t>
+          <t>Combined Confidence: 83688252.0144 (8368825201.4%)</t>
         </is>
       </c>
     </row>
@@ -2349,12 +2349,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
@@ -2391,12 +2391,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2416,7 +2416,7 @@
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -2433,23 +2433,23 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
@@ -2475,12 +2475,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -2500,7 +2500,7 @@
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>93.3</v>
+        <v>94.3</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Combined Confidence: 82410541.8825 (8241054188.2%)</t>
+          <t>Combined Confidence: 83155771.0896 (8315577109.0%)</t>
         </is>
       </c>
     </row>
@@ -2582,12 +2582,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
@@ -2624,12 +2624,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
@@ -2666,23 +2666,23 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
@@ -2708,23 +2708,23 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Wyatt Johnston</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>92.3</v>
+        <v>93.7</v>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Combined Confidence: 81696257.6625 (8169625766.2%)</t>
+          <t>Combined Confidence: 82800783.8064 (8280078380.6%)</t>
         </is>
       </c>
     </row>
@@ -2815,12 +2815,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
@@ -2840,7 +2840,7 @@
         </is>
       </c>
       <c r="H20" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
@@ -2857,12 +2857,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr"/>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -2882,7 +2882,7 @@
         </is>
       </c>
       <c r="H21" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
@@ -2899,23 +2899,23 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -2924,7 +2924,7 @@
         </is>
       </c>
       <c r="H22" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
@@ -2941,23 +2941,23 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Seth Jarvis</t>
+          <t>Tage Thompson</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="H23" s="4" t="n">
-        <v>91.5</v>
+        <v>93.3</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Combined Confidence: 81696257.6625 (8169625766.2%)</t>
+          <t>Combined Confidence: 81939281.2304 (8193928123.0%)</t>
         </is>
       </c>
     </row>
@@ -3048,12 +3048,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr"/>
@@ -3073,7 +3073,7 @@
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
@@ -3090,12 +3090,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -3115,7 +3115,7 @@
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
@@ -3132,23 +3132,23 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="H29" s="4" t="n">
-        <v>94.7</v>
+        <v>94.3</v>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
@@ -3174,12 +3174,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Kirill Kaprizov</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr"/>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>91.5</v>
+        <v>93.7</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Combined Confidence: 81696257.6625 (8169625766.2%)</t>
+          <t>Combined Confidence: 81853749.6216 (8185374962.2%)</t>
         </is>
       </c>
     </row>
@@ -3281,12 +3281,12 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
         </is>
       </c>
       <c r="H34" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
@@ -3323,12 +3323,12 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr"/>
@@ -3348,7 +3348,7 @@
         </is>
       </c>
       <c r="H35" s="4" t="n">
-        <v>96.7</v>
+        <v>95.7</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
@@ -3365,23 +3365,23 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="H36" s="4" t="n">
-        <v>94.7</v>
+        <v>94.3</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
@@ -3407,18 +3407,18 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Devon Toews</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -3432,7 +3432,7 @@
         </is>
       </c>
       <c r="H37" s="4" t="n">
-        <v>91.5</v>
+        <v>93.7</v>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
@@ -3474,7 +3474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-06 22:09 UTC</t>
+          <t>Generated: 2026-03-07 17:17 UTC</t>
         </is>
       </c>
     </row>
@@ -3487,7 +3487,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Combined Confidence: 7688903557.6372 (768890355763.7%)</t>
+          <t>Combined Confidence: 7841589213.7493 (784158921374.9%)</t>
         </is>
       </c>
     </row>
@@ -3551,12 +3551,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
@@ -3576,7 +3576,7 @@
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
@@ -3593,12 +3593,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
@@ -3635,23 +3635,23 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -3660,7 +3660,7 @@
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
@@ -3677,12 +3677,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -3702,7 +3702,7 @@
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>93.3</v>
+        <v>94.3</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
@@ -3719,23 +3719,23 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Wyatt Johnston</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -3744,7 +3744,7 @@
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>92.3</v>
+        <v>93.7</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Combined Confidence: 7622260839.9113 (762226083991.1%)</t>
+          <t>Combined Confidence: 7808113912.9435 (780811391294.4%)</t>
         </is>
       </c>
     </row>
@@ -3826,12 +3826,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
@@ -3851,7 +3851,7 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
@@ -3868,12 +3868,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr"/>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
@@ -3910,23 +3910,23 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -3935,7 +3935,7 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
@@ -3952,12 +3952,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Cole Perfetti</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr"/>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -3977,7 +3977,7 @@
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>93.3</v>
+        <v>94.3</v>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
@@ -3994,23 +3994,23 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Seth Jarvis</t>
+          <t>Tage Thompson</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -4019,7 +4019,7 @@
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>91.5</v>
+        <v>93.3</v>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Combined Confidence: 7622260839.9113 (762226083991.1%)</t>
+          <t>Combined Confidence: 7758433442.6597 (775843344266.0%)</t>
         </is>
       </c>
     </row>
@@ -4101,12 +4101,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Connor McDavid</t>
+          <t>Dougie Hamilton</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
@@ -4126,7 +4126,7 @@
         </is>
       </c>
       <c r="H22" s="4" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
@@ -4143,12 +4143,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Matthew Tkachuk</t>
+          <t>Mike Matheson</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -4168,7 +4168,7 @@
         </is>
       </c>
       <c r="H23" s="4" t="n">
-        <v>96.7</v>
+        <v>95.8</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
@@ -4185,23 +4185,23 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Matt Boldy</t>
+          <t>Nico Hischier</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NJ</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>POINTS</t>
+          <t>SHOTS ON GOAL</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -4210,7 +4210,7 @@
         </is>
       </c>
       <c r="H24" s="4" t="n">
-        <v>94.7</v>
+        <v>95.7</v>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
@@ -4227,18 +4227,18 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Gustav Forsling</t>
+          <t>Zach Werenski</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>SHOTS ON GOAL</t>
+          <t>POINTS</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -4252,7 +4252,7 @@
         </is>
       </c>
       <c r="H25" s="4" t="n">
-        <v>93.3</v>
+        <v>93.7</v>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
@@ -4269,12 +4269,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Kirill Kaprizov</t>
+          <t>Tage Thompson</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
@@ -4294,7 +4294,7 @@
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>91.5</v>
+        <v>93.3</v>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>

</xml_diff>